<commit_message>
Structure filter hide option
</commit_message>
<xml_diff>
--- a/Tests/PROS Equal Structures.xlsx
+++ b/Tests/PROS Equal Structures.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://queensuca-my.sharepoint.com/personal/gs13_queensu_ca/Documents/Python/Projects/StructureRelations/tests/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\OneDrive - Queen's University\Python\Projects\StructureRelations\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="37" documentId="8_{A094106A-2A7E-4402-8328-A7F404902C5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{635A2D2D-A69C-41A5-AD5F-162A69B88D05}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20AE84C6-8085-4AF1-99DC-EE4FD7686F5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{319760DD-07A2-4066-AC9A-8A9A60E5EC86}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="13740" windowHeight="21120" firstSheet="1" activeTab="3" xr2:uid="{319760DD-07A2-4066-AC9A-8A9A60E5EC86}"/>
   </bookViews>
   <sheets>
     <sheet name="RTROI Identification Code" sheetId="1" r:id="rId1"/>
@@ -478,7 +478,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -493,6 +493,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -519,7 +525,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -530,22 +536,19 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Bad" xfId="2" builtinId="27"/>
@@ -555,6 +558,9 @@
   <dxfs count="9">
     <dxf>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <border diagonalUp="0" diagonalDown="0">
@@ -567,6 +573,12 @@
         <vertical/>
         <horizontal/>
       </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -589,15 +601,6 @@
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -612,22 +615,22 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{79930D59-C53C-4751-A252-A367AD3CAEA3}" name="Table1" displayName="Table1" ref="A1:L32" totalsRowShown="0" headerRowDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{79930D59-C53C-4751-A252-A367AD3CAEA3}" name="Table1" displayName="Table1" ref="A1:L32" totalsRowShown="0" headerRowDxfId="5">
   <autoFilter ref="A1:L32" xr:uid="{79930D59-C53C-4751-A252-A367AD3CAEA3}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I32">
     <sortCondition ref="A13:A32"/>
   </sortState>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{6F97F3C7-FA2A-415C-BE90-C77E4D5EB9FD}" name="(3006,0084) _x000a_Referenced ROI Number"/>
-    <tableColumn id="2" xr3:uid="{75BD9A8E-764F-4B9A-A9FF-6E45CD31C674}" name="(0008,0100) _x000a_Code Value" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{75BD9A8E-764F-4B9A-A9FF-6E45CD31C674}" name="(0008,0100) _x000a_Code Value" dataDxfId="4"/>
     <tableColumn id="3" xr3:uid="{973AA4F2-4D6E-4581-ADED-563400401C3A}" name="(0008,0102) _x000a_Coding Scheme Designator"/>
-    <tableColumn id="4" xr3:uid="{317A4C95-9A7D-4D1D-9ED3-8B358CE619B3}" name="(0008,0103) _x000a_Coding Scheme Version" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{317A4C95-9A7D-4D1D-9ED3-8B358CE619B3}" name="(0008,0103) _x000a_Coding Scheme Version" dataDxfId="3"/>
     <tableColumn id="5" xr3:uid="{462B16AE-75C7-41AA-810F-9CC6A7C3E4D8}" name="(0008,0104) _x000a_Code Meaning"/>
     <tableColumn id="6" xr3:uid="{F501D714-24F8-4893-A12D-C067FB2E2EDA}" name="(3006,0088) _x000a_ROI Observation Description"/>
     <tableColumn id="7" xr3:uid="{DADB75C4-847A-4ED0-92E1-6C732CECDA43}" name="(3006,00A4) _x000a_RTROI Interpreted Type"/>
     <tableColumn id="8" xr3:uid="{9ECE9F98-984E-45AC-8108-F913ADB13EB4}" name="(3006,00B2) _x000a_ROI Physical Property"/>
     <tableColumn id="9" xr3:uid="{E6653436-2D09-4A5F-911E-2D84415C3171}" name="(3006,00B4) ROI _x000a_Physical Property Value"/>
-    <tableColumn id="10" xr3:uid="{239DC1EE-1100-430F-809B-1568E751E515}" name="(3006,0026) _x000a_ROI Name" dataDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{239DC1EE-1100-430F-809B-1568E751E515}" name="(3006,0026) _x000a_ROI Name" dataDxfId="2"/>
     <tableColumn id="11" xr3:uid="{F55E4290-17C4-4C50-913D-DFD216700DA7}" name="(3006,0036) _x000a_ROI Generation Algorithm"/>
     <tableColumn id="12" xr3:uid="{3E71568E-E584-4AC8-895A-CE2144BE9D9F}" name="(3006,0038) _x000a_ROI Generation Description"/>
   </tableColumns>
@@ -636,13 +639,13 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{47B5DDF6-F831-4662-9290-C3A3A0929E18}" name="Table2" displayName="Table2" ref="A2:D33" totalsRowShown="0" headerRowDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{47B5DDF6-F831-4662-9290-C3A3A0929E18}" name="Table2" displayName="Table2" ref="A2:D33" totalsRowShown="0" headerRowDxfId="1">
   <autoFilter ref="A2:D33" xr:uid="{47B5DDF6-F831-4662-9290-C3A3A0929E18}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:D33">
     <sortCondition ref="A6:A33"/>
   </sortState>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{DAD7D101-0D3B-4DC6-A722-6D4F7D4D31BE}" name="(3006,0022) _x000a_ROI Number" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{DAD7D101-0D3B-4DC6-A722-6D4F7D4D31BE}" name="(3006,0022) _x000a_ROI Number" dataDxfId="0"/>
     <tableColumn id="2" xr3:uid="{7FD546E2-B760-40A7-8C96-8BA2AE7D4A0C}" name="(3006,0026) _x000a_ROI Name"/>
     <tableColumn id="3" xr3:uid="{B6AF4AEC-9B66-4982-A157-A26FE85FF2A5}" name="(3006,0036) _x000a_ROI Generation Algorithm"/>
     <tableColumn id="4" xr3:uid="{0FD5D74C-DAF0-4DAD-93DB-299391C84950}" name="(3006,0038) _x000a_ROI Generation Description"/>
@@ -667,16 +670,16 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{CDE1D1E4-9556-41C4-991D-5D684DFC42B6}" name="Table15" displayName="Table15" ref="A1:E32" totalsRowShown="0" headerRowDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{CDE1D1E4-9556-41C4-991D-5D684DFC42B6}" name="Table15" displayName="Table15" ref="A1:E32" totalsRowShown="0" headerRowDxfId="8">
   <autoFilter ref="A1:E32" xr:uid="{79930D59-C53C-4751-A252-A367AD3CAEA3}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C32">
     <sortCondition ref="A13:A32"/>
   </sortState>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{558EAD63-78B6-40D8-850D-7C2C8BFD461F}" name="(3006,0084) _x000a_Referenced ROI Number" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{558EAD63-78B6-40D8-850D-7C2C8BFD461F}" name="(3006,0084) _x000a_Referenced ROI Number" dataDxfId="7"/>
     <tableColumn id="5" xr3:uid="{77816470-5310-4B89-9444-6ED80BA95371}" name="(0008,0104) _x000a_Code Meaning"/>
     <tableColumn id="7" xr3:uid="{84A58790-7996-4CF6-9187-2ED9498FC42B}" name="(3006,00A4) _x000a_RTROI Interpreted Type"/>
-    <tableColumn id="10" xr3:uid="{C9E4AD28-2176-40E0-923A-748043D86587}" name="(3006,0026) _x000a_ROI Name" dataDxfId="1"/>
+    <tableColumn id="10" xr3:uid="{C9E4AD28-2176-40E0-923A-748043D86587}" name="(3006,0026) _x000a_ROI Name" dataDxfId="6"/>
     <tableColumn id="13" xr3:uid="{C32D4786-23F7-4C49-9FA6-163EE97AE60E}" name="Matching Rule"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1060,13 +1063,13 @@
       <c r="I1" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="K1" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="L1" s="7" t="s">
+      <c r="L1" s="1" t="s">
         <v>103</v>
       </c>
     </row>
@@ -1089,13 +1092,13 @@
       <c r="F2" t="s">
         <v>12</v>
       </c>
-      <c r="J2" s="8" t="s">
+      <c r="J2" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="K2" s="9" t="s">
+      <c r="K2" t="s">
         <v>75</v>
       </c>
-      <c r="L2" s="9" t="s">
+      <c r="L2" t="s">
         <v>76</v>
       </c>
     </row>
@@ -1118,13 +1121,13 @@
       <c r="F3" t="s">
         <v>12</v>
       </c>
-      <c r="J3" s="8" t="s">
+      <c r="J3" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="K3" s="9" t="s">
+      <c r="K3" t="s">
         <v>75</v>
       </c>
-      <c r="L3" s="9" t="s">
+      <c r="L3" t="s">
         <v>76</v>
       </c>
     </row>
@@ -1147,13 +1150,12 @@
       <c r="F4" t="s">
         <v>16</v>
       </c>
-      <c r="J4" s="8" t="s">
+      <c r="J4" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="L4" s="9"/>
+      <c r="K4" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5">
@@ -1177,13 +1179,12 @@
       <c r="G5" t="s">
         <v>19</v>
       </c>
-      <c r="J5" s="8" t="s">
+      <c r="J5" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="K5" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="L5" s="9"/>
+      <c r="K5" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6">
@@ -1207,13 +1208,12 @@
       <c r="G6" t="s">
         <v>51</v>
       </c>
-      <c r="J6" s="8" t="s">
+      <c r="J6" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="K6" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="L6" s="9"/>
+      <c r="K6" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7">
@@ -1237,13 +1237,12 @@
       <c r="G7" t="s">
         <v>51</v>
       </c>
-      <c r="J7" s="8" t="s">
+      <c r="J7" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="K7" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="L7" s="9"/>
+      <c r="K7" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8">
@@ -1267,13 +1266,12 @@
       <c r="G8" t="s">
         <v>47</v>
       </c>
-      <c r="J8" s="8" t="s">
+      <c r="J8" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="K8" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="L8" s="9"/>
+      <c r="K8" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9">
@@ -1297,13 +1295,12 @@
       <c r="G9" t="s">
         <v>30</v>
       </c>
-      <c r="J9" s="8" t="s">
+      <c r="J9" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="K9" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="L9" s="9"/>
+      <c r="K9" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10">
@@ -1327,13 +1324,12 @@
       <c r="G10" t="s">
         <v>30</v>
       </c>
-      <c r="J10" s="8" t="s">
+      <c r="J10" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="K10" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="L10" s="9"/>
+      <c r="K10" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11">
@@ -1357,13 +1353,12 @@
       <c r="G11" t="s">
         <v>30</v>
       </c>
-      <c r="J11" s="8" t="s">
+      <c r="J11" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="K11" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="L11" s="9"/>
+      <c r="K11" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12">
@@ -1387,13 +1382,12 @@
       <c r="G12" t="s">
         <v>30</v>
       </c>
-      <c r="J12" s="8" t="s">
+      <c r="J12" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="K12" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="L12" s="9"/>
+      <c r="K12" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13">
@@ -1417,13 +1411,12 @@
       <c r="G13" t="s">
         <v>30</v>
       </c>
-      <c r="J13" s="8" t="s">
+      <c r="J13" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="K13" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="L13" s="9"/>
+      <c r="K13" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14">
@@ -1447,13 +1440,12 @@
       <c r="G14" t="s">
         <v>30</v>
       </c>
-      <c r="J14" s="8" t="s">
+      <c r="J14" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="K14" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="L14" s="9"/>
+      <c r="K14" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15">
@@ -1477,13 +1469,12 @@
       <c r="G15" t="s">
         <v>30</v>
       </c>
-      <c r="J15" s="8" t="s">
+      <c r="J15" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="K15" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="L15" s="9"/>
+      <c r="K15" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16">
@@ -1507,15 +1498,14 @@
       <c r="G16" t="s">
         <v>30</v>
       </c>
-      <c r="J16" s="8" t="s">
+      <c r="J16" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="K16" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="L16" s="9"/>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K16" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>32</v>
       </c>
@@ -1537,15 +1527,14 @@
       <c r="G17" t="s">
         <v>30</v>
       </c>
-      <c r="J17" s="8" t="s">
+      <c r="J17" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="K17" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="L17" s="9"/>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K17" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>33</v>
       </c>
@@ -1567,15 +1556,14 @@
       <c r="G18" t="s">
         <v>30</v>
       </c>
-      <c r="J18" s="8" t="s">
+      <c r="J18" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="K18" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="L18" s="9"/>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K18" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>34</v>
       </c>
@@ -1597,15 +1585,14 @@
       <c r="G19" t="s">
         <v>3</v>
       </c>
-      <c r="J19" s="8" t="s">
+      <c r="J19" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="K19" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="L19" s="9"/>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K19" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>35</v>
       </c>
@@ -1627,15 +1614,14 @@
       <c r="G20" t="s">
         <v>3</v>
       </c>
-      <c r="J20" s="8" t="s">
+      <c r="J20" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="K20" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="L20" s="9"/>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K20" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>36</v>
       </c>
@@ -1657,15 +1643,14 @@
       <c r="G21" t="s">
         <v>12</v>
       </c>
-      <c r="J21" s="8" t="s">
+      <c r="J21" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="K21" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="L21" s="9"/>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K21" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>37</v>
       </c>
@@ -1687,15 +1672,14 @@
       <c r="G22" t="s">
         <v>12</v>
       </c>
-      <c r="J22" s="8" t="s">
+      <c r="J22" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="K22" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="L22" s="9"/>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K22" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>38</v>
       </c>
@@ -1717,15 +1701,14 @@
       <c r="G23" t="s">
         <v>12</v>
       </c>
-      <c r="J23" s="8" t="s">
+      <c r="J23" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="K23" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="L23" s="9"/>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K23" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>42</v>
       </c>
@@ -1747,15 +1730,14 @@
       <c r="G24" t="s">
         <v>12</v>
       </c>
-      <c r="J24" s="8" t="s">
+      <c r="J24" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="K24" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="L24" s="9"/>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K24" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>44</v>
       </c>
@@ -1774,15 +1756,14 @@
       <c r="F25" t="s">
         <v>10</v>
       </c>
-      <c r="J25" s="8" t="s">
+      <c r="J25" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="K25" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="L25" s="9"/>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K25" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>45</v>
       </c>
@@ -1801,15 +1782,14 @@
       <c r="F26" t="s">
         <v>10</v>
       </c>
-      <c r="J26" s="8" t="s">
+      <c r="J26" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="K26" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="L26" s="9"/>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K26" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>46</v>
       </c>
@@ -1828,15 +1808,14 @@
       <c r="F27" t="s">
         <v>10</v>
       </c>
-      <c r="J27" s="8" t="s">
+      <c r="J27" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="K27" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="L27" s="9"/>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K27" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>47</v>
       </c>
@@ -1858,15 +1837,14 @@
       <c r="G28" t="s">
         <v>3</v>
       </c>
-      <c r="J28" s="8" t="s">
+      <c r="J28" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="K28" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="L28" s="9"/>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K28" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>48</v>
       </c>
@@ -1888,15 +1866,14 @@
       <c r="G29" t="s">
         <v>3</v>
       </c>
-      <c r="J29" s="8" t="s">
+      <c r="J29" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="K29" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="L29" s="9"/>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K29" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>49</v>
       </c>
@@ -1924,15 +1901,14 @@
       <c r="I30">
         <v>0.67705064655171998</v>
       </c>
-      <c r="J30" s="8" t="s">
+      <c r="J30" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="K30" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="L30" s="9"/>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K30" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>50</v>
       </c>
@@ -1960,15 +1936,14 @@
       <c r="I31">
         <v>1.0096525096499999E-3</v>
       </c>
-      <c r="J31" s="8" t="s">
+      <c r="J31" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="K31" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="L31" s="9"/>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K31" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>51</v>
       </c>
@@ -1990,13 +1965,12 @@
       <c r="G32" t="s">
         <v>30</v>
       </c>
-      <c r="J32" s="8" t="s">
+      <c r="J32" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="K32" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="L32" s="9"/>
+      <c r="K32" t="s">
+        <v>70</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2018,12 +1992,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
     </row>
     <row r="2" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
@@ -2413,15 +2387,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
@@ -2459,13 +2433,13 @@
       <c r="D3" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="F3" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="G3" s="6" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2560,7 +2534,7 @@
       <c r="C1" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="4" t="s">
         <v>101</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -2598,7 +2572,7 @@
       <c r="D2" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="E2" s="10" t="s">
+      <c r="E2" s="6" t="s">
         <v>112</v>
       </c>
       <c r="G2" t="s">
@@ -2613,13 +2587,13 @@
       <c r="J2" t="s">
         <v>11</v>
       </c>
-      <c r="K2" s="10" t="s">
+      <c r="K2" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="L2" s="10" t="s">
+      <c r="L2" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="M2" s="10" t="s">
+      <c r="M2" s="6" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2630,7 +2604,7 @@
       <c r="B3" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="5" t="s">
         <v>77</v>
       </c>
       <c r="G3" t="s">
@@ -2653,7 +2627,7 @@
       <c r="B4" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="5" t="s">
         <v>14</v>
       </c>
       <c r="G4" t="s">
@@ -2688,7 +2662,7 @@
       <c r="C5" t="s">
         <v>19</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="5" t="s">
         <v>78</v>
       </c>
       <c r="G5" t="s">
@@ -2714,7 +2688,7 @@
       <c r="C6" t="s">
         <v>51</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="5" t="s">
         <v>96</v>
       </c>
     </row>
@@ -2728,7 +2702,7 @@
       <c r="C7" t="s">
         <v>51</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="5" t="s">
         <v>95</v>
       </c>
     </row>
@@ -2742,7 +2716,7 @@
       <c r="C8" t="s">
         <v>47</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="5" t="s">
         <v>44</v>
       </c>
     </row>
@@ -2759,7 +2733,7 @@
       <c r="D9" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="E9" s="11" t="s">
+      <c r="E9" s="7" t="s">
         <v>122</v>
       </c>
     </row>
@@ -2776,7 +2750,7 @@
       <c r="D10" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="E10" s="11" t="s">
+      <c r="E10" s="7" t="s">
         <v>122</v>
       </c>
     </row>
@@ -2793,7 +2767,7 @@
       <c r="D11" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="E11" s="11" t="s">
+      <c r="E11" s="7" t="s">
         <v>122</v>
       </c>
     </row>
@@ -2807,7 +2781,7 @@
       <c r="C12" t="s">
         <v>30</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="D12" s="5" t="s">
         <v>91</v>
       </c>
     </row>
@@ -2821,7 +2795,7 @@
       <c r="C13" t="s">
         <v>30</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="5" t="s">
         <v>90</v>
       </c>
     </row>
@@ -2835,7 +2809,7 @@
       <c r="C14" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="5" t="s">
         <v>89</v>
       </c>
     </row>
@@ -2849,7 +2823,7 @@
       <c r="C15" t="s">
         <v>30</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" s="5" t="s">
         <v>88</v>
       </c>
     </row>
@@ -2863,7 +2837,7 @@
       <c r="C16" t="s">
         <v>30</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="D16" s="5" t="s">
         <v>87</v>
       </c>
     </row>
@@ -2877,7 +2851,7 @@
       <c r="C17" t="s">
         <v>30</v>
       </c>
-      <c r="D17" s="8" t="s">
+      <c r="D17" s="5" t="s">
         <v>86</v>
       </c>
     </row>
@@ -2891,7 +2865,7 @@
       <c r="C18" t="s">
         <v>30</v>
       </c>
-      <c r="D18" s="8" t="s">
+      <c r="D18" s="5" t="s">
         <v>85</v>
       </c>
     </row>
@@ -2908,7 +2882,7 @@
       <c r="D19" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="E19" s="11" t="s">
+      <c r="E19" s="7" t="s">
         <v>120</v>
       </c>
     </row>
@@ -2925,7 +2899,7 @@
       <c r="D20" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="E20" s="11" t="s">
+      <c r="E20" s="7" t="s">
         <v>120</v>
       </c>
     </row>
@@ -2939,7 +2913,7 @@
       <c r="C21" t="s">
         <v>12</v>
       </c>
-      <c r="D21" s="8" t="s">
+      <c r="D21" s="5" t="s">
         <v>82</v>
       </c>
     </row>
@@ -2953,7 +2927,7 @@
       <c r="C22" t="s">
         <v>12</v>
       </c>
-      <c r="D22" s="8" t="s">
+      <c r="D22" s="5" t="s">
         <v>81</v>
       </c>
     </row>
@@ -2967,7 +2941,7 @@
       <c r="C23" t="s">
         <v>12</v>
       </c>
-      <c r="D23" s="8" t="s">
+      <c r="D23" s="5" t="s">
         <v>80</v>
       </c>
     </row>
@@ -2981,7 +2955,7 @@
       <c r="C24" t="s">
         <v>12</v>
       </c>
-      <c r="D24" s="8" t="s">
+      <c r="D24" s="5" t="s">
         <v>1</v>
       </c>
     </row>
@@ -2995,7 +2969,7 @@
       <c r="D25" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="E25" s="11" t="s">
+      <c r="E25" s="7" t="s">
         <v>116</v>
       </c>
     </row>
@@ -3009,7 +2983,7 @@
       <c r="D26" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="E26" s="11" t="s">
+      <c r="E26" s="7" t="s">
         <v>116</v>
       </c>
     </row>
@@ -3023,7 +2997,7 @@
       <c r="D27" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="E27" s="11" t="s">
+      <c r="E27" s="7" t="s">
         <v>116</v>
       </c>
     </row>
@@ -3037,7 +3011,7 @@
       <c r="C28" t="s">
         <v>3</v>
       </c>
-      <c r="D28" s="8" t="s">
+      <c r="D28" s="5" t="s">
         <v>71</v>
       </c>
     </row>
@@ -3051,7 +3025,7 @@
       <c r="C29" t="s">
         <v>3</v>
       </c>
-      <c r="D29" s="8" t="s">
+      <c r="D29" s="5" t="s">
         <v>69</v>
       </c>
     </row>
@@ -3065,7 +3039,7 @@
       <c r="C30" t="s">
         <v>57</v>
       </c>
-      <c r="D30" s="8" t="s">
+      <c r="D30" s="5" t="s">
         <v>97</v>
       </c>
     </row>
@@ -3079,7 +3053,7 @@
       <c r="C31" t="s">
         <v>57</v>
       </c>
-      <c r="D31" s="8" t="s">
+      <c r="D31" s="5" t="s">
         <v>98</v>
       </c>
     </row>
@@ -3093,7 +3067,7 @@
       <c r="C32" t="s">
         <v>30</v>
       </c>
-      <c r="D32" s="8" t="s">
+      <c r="D32" s="5" t="s">
         <v>99</v>
       </c>
     </row>

</xml_diff>